<commit_message>
feat: add realistic synthetic risk dataset
</commit_message>
<xml_diff>
--- a/sample-data/MIS.xlsx
+++ b/sample-data/MIS.xlsx
@@ -1580,7 +1580,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1605,7 +1605,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1630,7 +1630,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>

</xml_diff>